<commit_message>
[FIX] Discriminateur Patient.contact.relationship via extension
Résolution de l'issue #290 : le discriminant $this avec binding extensible
n'est pas évaluable par les validateurs FHIR.

Solution retenue : ajout d'une extension fr-core-patient-contact-relationship-category
(code fixé par slice) comme discriminant déterministe.

- Ajout CodeSystem FRCoreCodeSystemPatientContactRelationshipCategory (#role, #relationType)
- Ajout ValueSet FRCoreValueSetPatientContactRelationshipCategory
- Ajout Extension FRCorePatientContactRelationshipCategoryExtension
- Mise à jour FRCorePatientProfile : discriminant sur l'extension, code fixé par slice
- Mise à jour FRCorePatientExample : ajout de l'extension sur chaque relationship

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> f81553e1c44740763c5e2b7961a0733475ec4094
</commit_message>
<xml_diff>
--- a/nr-update-patient-relationship-discr/ig/StructureDefinition-fr-core-patient-ins.xlsx
+++ b/nr-update-patient-relationship-discr/ig/StructureDefinition-fr-core-patient-ins.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AO$214</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AO$232</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7952" uniqueCount="905">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8610" uniqueCount="952">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-20T07:02:57+00:00</t>
+    <t>2026-03-20T07:20:31+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2546,6 +2546,10 @@
     <t>http://hl7.org/fhir/ValueSet/patient-contactrelationship|4.0.1</t>
   </si>
   <si>
+    <t xml:space="preserve">value:extension('https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient-contact-relationship-category').value}
+</t>
+  </si>
+  <si>
     <t>code</t>
   </si>
   <si>
@@ -2564,6 +2568,118 @@
     <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-patient-contact-role|2.2.0-ballot-2</t>
   </si>
   <si>
+    <t>Patient.contact.relationship:role.id</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship.id</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:role.extension</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship.extension</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:role.extension:category</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient-contact-relationship-category|2.2.0-ballot-2}
+</t>
+  </si>
+  <si>
+    <t>FR Core Patient Contact Relationship Category Extension</t>
+  </si>
+  <si>
+    <t>Catégorie de la relation du contact patient : indique si le CodeableConcept représente un rôle (ex : personne à prévenir) ou un type de relation (ex : mère)</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:role.extension:category.id</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship.extension.id</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:role.extension:category.extension</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship.extension.extension</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:role.extension:category.url</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship.extension.url</t>
+  </si>
+  <si>
+    <t>https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient-contact-relationship-category</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:role.extension:category.value[x]</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship.extension.value[x]</t>
+  </si>
+  <si>
+    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-patient-contact-relationship-category|2.2.0-ballot-2</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:role.coding</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship.coding</t>
+  </si>
+  <si>
+    <t>Code defined by a terminology system</t>
+  </si>
+  <si>
+    <t>A reference to a code defined by a terminology system.</t>
+  </si>
+  <si>
+    <t>Codes may be defined very casually in enumerations, or code lists, up to very formal definitions such as SNOMED CT - see the HL7 v3 Core Principles for more information.  Ordering of codings is undefined and SHALL NOT be used to infer meaning. Generally, at most only one of the coding values will be labeled as UserSelected = true.</t>
+  </si>
+  <si>
+    <t>Allows for alternative encodings within a code system, and translations to other code systems.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.coding</t>
+  </si>
+  <si>
+    <t>union(., ./translation)</t>
+  </si>
+  <si>
+    <t>C*E.1-8, C*E.10-22</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:role.text</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship.text</t>
+  </si>
+  <si>
+    <t>Plain text representation of the concept</t>
+  </si>
+  <si>
+    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
+  </si>
+  <si>
+    <t>Very often the text is the same as a displayName of one of the codings.</t>
+  </si>
+  <si>
+    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.text</t>
+  </si>
+  <si>
+    <t>./originalText[mediaType/code="text/plain"]/data</t>
+  </si>
+  <si>
+    <t>C*E.9. But note many systems use C*E.2 for this</t>
+  </si>
+  <si>
     <t>Patient.contact.relationship:relationType</t>
   </si>
   <si>
@@ -2574,6 +2690,33 @@
   </si>
   <si>
     <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-relation-type|2.2.0-ballot-2</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:relationType.id</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:relationType.extension</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:relationType.extension:category</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:relationType.extension:category.id</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:relationType.extension:category.extension</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:relationType.extension:category.url</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:relationType.extension:category.value[x]</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:relationType.coding</t>
+  </si>
+  <si>
+    <t>Patient.contact.relationship:relationType.text</t>
   </si>
   <si>
     <t>Patient.contact.name</t>
@@ -3193,11 +3336,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AO214"/>
+  <dimension ref="A1:AO232"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="59.65625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="33.83984375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="38.97265625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="20.984375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="34.21875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -3221,9 +3364,9 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="84.54296875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="69.14453125" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="76.39453125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="91.3359375" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="64.65625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
@@ -25644,7 +25787,7 @@
         <v>82</v>
       </c>
       <c r="AB192" t="s" s="2">
-        <v>142</v>
+        <v>800</v>
       </c>
       <c r="AC192" s="2"/>
       <c r="AD192" t="s" s="2">
@@ -25669,7 +25812,7 @@
         <v>102</v>
       </c>
       <c r="AK192" t="s" s="2">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="AL192" t="s" s="2">
         <v>108</v>
@@ -25678,7 +25821,7 @@
         <v>82</v>
       </c>
       <c r="AN192" t="s" s="2">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="AO192" t="s" s="2">
         <v>82</v>
@@ -25686,13 +25829,13 @@
     </row>
     <row r="193" hidden="true">
       <c r="A193" t="s" s="2">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="B193" t="s" s="2">
         <v>794</v>
       </c>
       <c r="C193" t="s" s="2">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="D193" t="s" s="2">
         <v>82</v>
@@ -25717,7 +25860,7 @@
         <v>439</v>
       </c>
       <c r="L193" t="s" s="2">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="M193" t="s" s="2">
         <v>796</v>
@@ -25753,7 +25896,7 @@
       </c>
       <c r="Y193" s="2"/>
       <c r="Z193" t="s" s="2">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="AA193" t="s" s="2">
         <v>82</v>
@@ -25786,7 +25929,7 @@
         <v>102</v>
       </c>
       <c r="AK193" t="s" s="2">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="AL193" t="s" s="2">
         <v>108</v>
@@ -25795,7 +25938,7 @@
         <v>82</v>
       </c>
       <c r="AN193" t="s" s="2">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="AO193" t="s" s="2">
         <v>82</v>
@@ -25803,14 +25946,12 @@
     </row>
     <row r="194" hidden="true">
       <c r="A194" t="s" s="2">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="B194" t="s" s="2">
-        <v>794</v>
-      </c>
-      <c r="C194" t="s" s="2">
-        <v>807</v>
-      </c>
+        <v>808</v>
+      </c>
+      <c r="C194" s="2"/>
       <c r="D194" t="s" s="2">
         <v>82</v>
       </c>
@@ -25831,18 +25972,16 @@
         <v>82</v>
       </c>
       <c r="K194" t="s" s="2">
-        <v>439</v>
+        <v>104</v>
       </c>
       <c r="L194" t="s" s="2">
-        <v>808</v>
+        <v>105</v>
       </c>
       <c r="M194" t="s" s="2">
-        <v>796</v>
+        <v>106</v>
       </c>
       <c r="N194" s="2"/>
-      <c r="O194" t="s" s="2">
-        <v>797</v>
-      </c>
+      <c r="O194" s="2"/>
       <c r="P194" t="s" s="2">
         <v>82</v>
       </c>
@@ -25866,11 +26005,13 @@
         <v>82</v>
       </c>
       <c r="X194" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="Y194" s="2"/>
+        <v>82</v>
+      </c>
+      <c r="Y194" t="s" s="2">
+        <v>82</v>
+      </c>
       <c r="Z194" t="s" s="2">
-        <v>809</v>
+        <v>82</v>
       </c>
       <c r="AA194" t="s" s="2">
         <v>82</v>
@@ -25888,31 +26029,31 @@
         <v>82</v>
       </c>
       <c r="AF194" t="s" s="2">
-        <v>794</v>
+        <v>107</v>
       </c>
       <c r="AG194" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH194" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI194" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ194" t="s" s="2">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="AK194" t="s" s="2">
-        <v>800</v>
+        <v>108</v>
       </c>
       <c r="AL194" t="s" s="2">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="AM194" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN194" t="s" s="2">
-        <v>801</v>
+        <v>82</v>
       </c>
       <c r="AO194" t="s" s="2">
         <v>82</v>
@@ -25920,7 +26061,7 @@
     </row>
     <row r="195" hidden="true">
       <c r="A195" t="s" s="2">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="B195" t="s" s="2">
         <v>810</v>
@@ -25931,10 +26072,10 @@
       </c>
       <c r="E195" s="2"/>
       <c r="F195" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G195" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H195" t="s" s="2">
         <v>82</v>
@@ -25946,18 +26087,16 @@
         <v>82</v>
       </c>
       <c r="K195" t="s" s="2">
-        <v>608</v>
+        <v>111</v>
       </c>
       <c r="L195" t="s" s="2">
-        <v>811</v>
+        <v>198</v>
       </c>
       <c r="M195" t="s" s="2">
-        <v>812</v>
+        <v>199</v>
       </c>
       <c r="N195" s="2"/>
-      <c r="O195" t="s" s="2">
-        <v>813</v>
-      </c>
+      <c r="O195" s="2"/>
       <c r="P195" t="s" s="2">
         <v>82</v>
       </c>
@@ -25993,43 +26132,43 @@
         <v>82</v>
       </c>
       <c r="AB195" t="s" s="2">
-        <v>82</v>
+        <v>115</v>
       </c>
       <c r="AC195" t="s" s="2">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="AD195" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE195" t="s" s="2">
-        <v>82</v>
+        <v>117</v>
       </c>
       <c r="AF195" t="s" s="2">
-        <v>810</v>
+        <v>118</v>
       </c>
       <c r="AG195" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH195" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI195" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ195" t="s" s="2">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="AK195" t="s" s="2">
-        <v>614</v>
+        <v>82</v>
       </c>
       <c r="AL195" t="s" s="2">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="AM195" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN195" t="s" s="2">
-        <v>814</v>
+        <v>82</v>
       </c>
       <c r="AO195" t="s" s="2">
         <v>82</v>
@@ -26037,21 +26176,23 @@
     </row>
     <row r="196" hidden="true">
       <c r="A196" t="s" s="2">
-        <v>815</v>
+        <v>811</v>
       </c>
       <c r="B196" t="s" s="2">
-        <v>815</v>
-      </c>
-      <c r="C196" s="2"/>
+        <v>810</v>
+      </c>
+      <c r="C196" t="s" s="2">
+        <v>812</v>
+      </c>
       <c r="D196" t="s" s="2">
         <v>82</v>
       </c>
       <c r="E196" s="2"/>
       <c r="F196" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G196" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H196" t="s" s="2">
         <v>82</v>
@@ -26063,20 +26204,16 @@
         <v>82</v>
       </c>
       <c r="K196" t="s" s="2">
-        <v>703</v>
+        <v>813</v>
       </c>
       <c r="L196" t="s" s="2">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="M196" t="s" s="2">
-        <v>817</v>
-      </c>
-      <c r="N196" t="s" s="2">
-        <v>818</v>
-      </c>
-      <c r="O196" t="s" s="2">
-        <v>707</v>
-      </c>
+        <v>815</v>
+      </c>
+      <c r="N196" s="2"/>
+      <c r="O196" s="2"/>
       <c r="P196" t="s" s="2">
         <v>82</v>
       </c>
@@ -26124,7 +26261,7 @@
         <v>82</v>
       </c>
       <c r="AF196" t="s" s="2">
-        <v>815</v>
+        <v>118</v>
       </c>
       <c r="AG196" t="s" s="2">
         <v>80</v>
@@ -26136,19 +26273,19 @@
         <v>82</v>
       </c>
       <c r="AJ196" t="s" s="2">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="AK196" t="s" s="2">
-        <v>708</v>
+        <v>82</v>
       </c>
       <c r="AL196" t="s" s="2">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="AM196" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN196" t="s" s="2">
-        <v>819</v>
+        <v>82</v>
       </c>
       <c r="AO196" t="s" s="2">
         <v>82</v>
@@ -26156,10 +26293,10 @@
     </row>
     <row r="197" hidden="true">
       <c r="A197" t="s" s="2">
-        <v>820</v>
+        <v>816</v>
       </c>
       <c r="B197" t="s" s="2">
-        <v>820</v>
+        <v>817</v>
       </c>
       <c r="C197" s="2"/>
       <c r="D197" t="s" s="2">
@@ -26182,18 +26319,16 @@
         <v>82</v>
       </c>
       <c r="K197" t="s" s="2">
-        <v>821</v>
+        <v>104</v>
       </c>
       <c r="L197" t="s" s="2">
-        <v>822</v>
+        <v>105</v>
       </c>
       <c r="M197" t="s" s="2">
-        <v>823</v>
+        <v>106</v>
       </c>
       <c r="N197" s="2"/>
-      <c r="O197" t="s" s="2">
-        <v>824</v>
-      </c>
+      <c r="O197" s="2"/>
       <c r="P197" t="s" s="2">
         <v>82</v>
       </c>
@@ -26241,7 +26376,7 @@
         <v>82</v>
       </c>
       <c r="AF197" t="s" s="2">
-        <v>820</v>
+        <v>107</v>
       </c>
       <c r="AG197" t="s" s="2">
         <v>80</v>
@@ -26253,19 +26388,19 @@
         <v>82</v>
       </c>
       <c r="AJ197" t="s" s="2">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="AK197" t="s" s="2">
-        <v>742</v>
+        <v>108</v>
       </c>
       <c r="AL197" t="s" s="2">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="AM197" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN197" t="s" s="2">
-        <v>825</v>
+        <v>82</v>
       </c>
       <c r="AO197" t="s" s="2">
         <v>82</v>
@@ -26273,10 +26408,10 @@
     </row>
     <row r="198" hidden="true">
       <c r="A198" t="s" s="2">
-        <v>826</v>
+        <v>818</v>
       </c>
       <c r="B198" t="s" s="2">
-        <v>826</v>
+        <v>819</v>
       </c>
       <c r="C198" s="2"/>
       <c r="D198" t="s" s="2">
@@ -26287,7 +26422,7 @@
         <v>80</v>
       </c>
       <c r="G198" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H198" t="s" s="2">
         <v>82</v>
@@ -26299,18 +26434,16 @@
         <v>82</v>
       </c>
       <c r="K198" t="s" s="2">
-        <v>173</v>
+        <v>111</v>
       </c>
       <c r="L198" t="s" s="2">
-        <v>827</v>
+        <v>198</v>
       </c>
       <c r="M198" t="s" s="2">
-        <v>828</v>
+        <v>199</v>
       </c>
       <c r="N198" s="2"/>
-      <c r="O198" t="s" s="2">
-        <v>829</v>
-      </c>
+      <c r="O198" s="2"/>
       <c r="P198" t="s" s="2">
         <v>82</v>
       </c>
@@ -26334,55 +26467,55 @@
         <v>82</v>
       </c>
       <c r="X198" t="s" s="2">
-        <v>264</v>
+        <v>82</v>
       </c>
       <c r="Y198" t="s" s="2">
-        <v>830</v>
+        <v>82</v>
       </c>
       <c r="Z198" t="s" s="2">
-        <v>831</v>
+        <v>82</v>
       </c>
       <c r="AA198" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AB198" t="s" s="2">
-        <v>82</v>
+        <v>115</v>
       </c>
       <c r="AC198" t="s" s="2">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="AD198" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE198" t="s" s="2">
-        <v>82</v>
+        <v>117</v>
       </c>
       <c r="AF198" t="s" s="2">
-        <v>826</v>
+        <v>118</v>
       </c>
       <c r="AG198" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH198" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI198" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ198" t="s" s="2">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="AK198" t="s" s="2">
-        <v>717</v>
+        <v>82</v>
       </c>
       <c r="AL198" t="s" s="2">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="AM198" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN198" t="s" s="2">
-        <v>832</v>
+        <v>82</v>
       </c>
       <c r="AO198" t="s" s="2">
         <v>82</v>
@@ -26390,10 +26523,10 @@
     </row>
     <row r="199" hidden="true">
       <c r="A199" t="s" s="2">
-        <v>833</v>
+        <v>820</v>
       </c>
       <c r="B199" t="s" s="2">
-        <v>833</v>
+        <v>821</v>
       </c>
       <c r="C199" s="2"/>
       <c r="D199" t="s" s="2">
@@ -26401,7 +26534,7 @@
       </c>
       <c r="E199" s="2"/>
       <c r="F199" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G199" t="s" s="2">
         <v>90</v>
@@ -26416,24 +26549,24 @@
         <v>82</v>
       </c>
       <c r="K199" t="s" s="2">
-        <v>477</v>
+        <v>132</v>
       </c>
       <c r="L199" t="s" s="2">
-        <v>834</v>
+        <v>225</v>
       </c>
       <c r="M199" t="s" s="2">
-        <v>835</v>
-      </c>
-      <c r="N199" s="2"/>
-      <c r="O199" t="s" s="2">
-        <v>836</v>
-      </c>
+        <v>226</v>
+      </c>
+      <c r="N199" t="s" s="2">
+        <v>227</v>
+      </c>
+      <c r="O199" s="2"/>
       <c r="P199" t="s" s="2">
         <v>82</v>
       </c>
       <c r="Q199" s="2"/>
       <c r="R199" t="s" s="2">
-        <v>82</v>
+        <v>822</v>
       </c>
       <c r="S199" t="s" s="2">
         <v>82</v>
@@ -26475,31 +26608,31 @@
         <v>82</v>
       </c>
       <c r="AF199" t="s" s="2">
-        <v>833</v>
+        <v>228</v>
       </c>
       <c r="AG199" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AH199" t="s" s="2">
         <v>90</v>
       </c>
       <c r="AI199" t="s" s="2">
-        <v>837</v>
+        <v>82</v>
       </c>
       <c r="AJ199" t="s" s="2">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="AK199" t="s" s="2">
-        <v>838</v>
+        <v>196</v>
       </c>
       <c r="AL199" t="s" s="2">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="AM199" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN199" t="s" s="2">
-        <v>839</v>
+        <v>82</v>
       </c>
       <c r="AO199" t="s" s="2">
         <v>82</v>
@@ -26507,10 +26640,10 @@
     </row>
     <row r="200" hidden="true">
       <c r="A200" t="s" s="2">
-        <v>840</v>
+        <v>823</v>
       </c>
       <c r="B200" t="s" s="2">
-        <v>840</v>
+        <v>824</v>
       </c>
       <c r="C200" s="2"/>
       <c r="D200" t="s" s="2">
@@ -26533,13 +26666,13 @@
         <v>82</v>
       </c>
       <c r="K200" t="s" s="2">
-        <v>390</v>
+        <v>173</v>
       </c>
       <c r="L200" t="s" s="2">
-        <v>841</v>
+        <v>231</v>
       </c>
       <c r="M200" t="s" s="2">
-        <v>842</v>
+        <v>232</v>
       </c>
       <c r="N200" s="2"/>
       <c r="O200" s="2"/>
@@ -26551,7 +26684,7 @@
         <v>82</v>
       </c>
       <c r="S200" t="s" s="2">
-        <v>82</v>
+        <v>804</v>
       </c>
       <c r="T200" t="s" s="2">
         <v>82</v>
@@ -26566,13 +26699,11 @@
         <v>82</v>
       </c>
       <c r="X200" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y200" t="s" s="2">
-        <v>82</v>
-      </c>
+        <v>264</v>
+      </c>
+      <c r="Y200" s="2"/>
       <c r="Z200" t="s" s="2">
-        <v>82</v>
+        <v>825</v>
       </c>
       <c r="AA200" t="s" s="2">
         <v>82</v>
@@ -26590,7 +26721,7 @@
         <v>82</v>
       </c>
       <c r="AF200" t="s" s="2">
-        <v>840</v>
+        <v>234</v>
       </c>
       <c r="AG200" t="s" s="2">
         <v>80</v>
@@ -26605,10 +26736,10 @@
         <v>102</v>
       </c>
       <c r="AK200" t="s" s="2">
-        <v>843</v>
+        <v>196</v>
       </c>
       <c r="AL200" t="s" s="2">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="AM200" t="s" s="2">
         <v>82</v>
@@ -26622,10 +26753,10 @@
     </row>
     <row r="201" hidden="true">
       <c r="A201" t="s" s="2">
-        <v>844</v>
+        <v>826</v>
       </c>
       <c r="B201" t="s" s="2">
-        <v>844</v>
+        <v>827</v>
       </c>
       <c r="C201" s="2"/>
       <c r="D201" t="s" s="2">
@@ -26645,22 +26776,22 @@
         <v>82</v>
       </c>
       <c r="J201" t="s" s="2">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="K201" t="s" s="2">
-        <v>770</v>
+        <v>151</v>
       </c>
       <c r="L201" t="s" s="2">
-        <v>845</v>
+        <v>828</v>
       </c>
       <c r="M201" t="s" s="2">
-        <v>846</v>
+        <v>829</v>
       </c>
       <c r="N201" t="s" s="2">
-        <v>847</v>
+        <v>830</v>
       </c>
       <c r="O201" t="s" s="2">
-        <v>848</v>
+        <v>831</v>
       </c>
       <c r="P201" t="s" s="2">
         <v>82</v>
@@ -26709,7 +26840,7 @@
         <v>82</v>
       </c>
       <c r="AF201" t="s" s="2">
-        <v>844</v>
+        <v>832</v>
       </c>
       <c r="AG201" t="s" s="2">
         <v>80</v>
@@ -26724,16 +26855,16 @@
         <v>102</v>
       </c>
       <c r="AK201" t="s" s="2">
-        <v>849</v>
+        <v>833</v>
       </c>
       <c r="AL201" t="s" s="2">
-        <v>850</v>
+        <v>82</v>
       </c>
       <c r="AM201" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN201" t="s" s="2">
-        <v>82</v>
+        <v>834</v>
       </c>
       <c r="AO201" t="s" s="2">
         <v>82</v>
@@ -26741,10 +26872,10 @@
     </row>
     <row r="202" hidden="true">
       <c r="A202" t="s" s="2">
-        <v>851</v>
+        <v>835</v>
       </c>
       <c r="B202" t="s" s="2">
-        <v>851</v>
+        <v>836</v>
       </c>
       <c r="C202" s="2"/>
       <c r="D202" t="s" s="2">
@@ -26764,19 +26895,23 @@
         <v>82</v>
       </c>
       <c r="J202" t="s" s="2">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="K202" t="s" s="2">
         <v>104</v>
       </c>
       <c r="L202" t="s" s="2">
-        <v>105</v>
+        <v>837</v>
       </c>
       <c r="M202" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="N202" s="2"/>
-      <c r="O202" s="2"/>
+        <v>838</v>
+      </c>
+      <c r="N202" t="s" s="2">
+        <v>839</v>
+      </c>
+      <c r="O202" t="s" s="2">
+        <v>840</v>
+      </c>
       <c r="P202" t="s" s="2">
         <v>82</v>
       </c>
@@ -26824,7 +26959,7 @@
         <v>82</v>
       </c>
       <c r="AF202" t="s" s="2">
-        <v>107</v>
+        <v>841</v>
       </c>
       <c r="AG202" t="s" s="2">
         <v>80</v>
@@ -26836,10 +26971,10 @@
         <v>82</v>
       </c>
       <c r="AJ202" t="s" s="2">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="AK202" t="s" s="2">
-        <v>108</v>
+        <v>842</v>
       </c>
       <c r="AL202" t="s" s="2">
         <v>82</v>
@@ -26848,7 +26983,7 @@
         <v>82</v>
       </c>
       <c r="AN202" t="s" s="2">
-        <v>82</v>
+        <v>843</v>
       </c>
       <c r="AO202" t="s" s="2">
         <v>82</v>
@@ -26856,21 +26991,23 @@
     </row>
     <row r="203" hidden="true">
       <c r="A203" t="s" s="2">
-        <v>852</v>
+        <v>844</v>
       </c>
       <c r="B203" t="s" s="2">
-        <v>852</v>
-      </c>
-      <c r="C203" s="2"/>
+        <v>794</v>
+      </c>
+      <c r="C203" t="s" s="2">
+        <v>845</v>
+      </c>
       <c r="D203" t="s" s="2">
-        <v>110</v>
+        <v>82</v>
       </c>
       <c r="E203" s="2"/>
       <c r="F203" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G203" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H203" t="s" s="2">
         <v>82</v>
@@ -26882,18 +27019,18 @@
         <v>82</v>
       </c>
       <c r="K203" t="s" s="2">
-        <v>111</v>
+        <v>439</v>
       </c>
       <c r="L203" t="s" s="2">
-        <v>112</v>
+        <v>846</v>
       </c>
       <c r="M203" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N203" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="O203" s="2"/>
+        <v>796</v>
+      </c>
+      <c r="N203" s="2"/>
+      <c r="O203" t="s" s="2">
+        <v>797</v>
+      </c>
       <c r="P203" t="s" s="2">
         <v>82</v>
       </c>
@@ -26917,13 +27054,11 @@
         <v>82</v>
       </c>
       <c r="X203" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y203" t="s" s="2">
-        <v>82</v>
-      </c>
+        <v>155</v>
+      </c>
+      <c r="Y203" s="2"/>
       <c r="Z203" t="s" s="2">
-        <v>82</v>
+        <v>847</v>
       </c>
       <c r="AA203" t="s" s="2">
         <v>82</v>
@@ -26941,7 +27076,7 @@
         <v>82</v>
       </c>
       <c r="AF203" t="s" s="2">
-        <v>118</v>
+        <v>794</v>
       </c>
       <c r="AG203" t="s" s="2">
         <v>80</v>
@@ -26953,19 +27088,19 @@
         <v>82</v>
       </c>
       <c r="AJ203" t="s" s="2">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="AK203" t="s" s="2">
+        <v>801</v>
+      </c>
+      <c r="AL203" t="s" s="2">
         <v>108</v>
       </c>
-      <c r="AL203" t="s" s="2">
-        <v>82</v>
-      </c>
       <c r="AM203" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN203" t="s" s="2">
-        <v>82</v>
+        <v>802</v>
       </c>
       <c r="AO203" t="s" s="2">
         <v>82</v>
@@ -26973,46 +27108,42 @@
     </row>
     <row r="204" hidden="true">
       <c r="A204" t="s" s="2">
-        <v>853</v>
+        <v>848</v>
       </c>
       <c r="B204" t="s" s="2">
-        <v>853</v>
+        <v>808</v>
       </c>
       <c r="C204" s="2"/>
       <c r="D204" t="s" s="2">
-        <v>790</v>
+        <v>82</v>
       </c>
       <c r="E204" s="2"/>
       <c r="F204" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G204" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H204" t="s" s="2">
         <v>82</v>
       </c>
       <c r="I204" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="J204" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="K204" t="s" s="2">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="L204" t="s" s="2">
-        <v>791</v>
+        <v>105</v>
       </c>
       <c r="M204" t="s" s="2">
-        <v>792</v>
-      </c>
-      <c r="N204" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="O204" t="s" s="2">
-        <v>406</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="N204" s="2"/>
+      <c r="O204" s="2"/>
       <c r="P204" t="s" s="2">
         <v>82</v>
       </c>
@@ -27060,22 +27191,22 @@
         <v>82</v>
       </c>
       <c r="AF204" t="s" s="2">
-        <v>793</v>
+        <v>107</v>
       </c>
       <c r="AG204" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH204" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI204" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ204" t="s" s="2">
-        <v>119</v>
+        <v>82</v>
       </c>
       <c r="AK204" t="s" s="2">
-        <v>196</v>
+        <v>108</v>
       </c>
       <c r="AL204" t="s" s="2">
         <v>82</v>
@@ -27092,10 +27223,10 @@
     </row>
     <row r="205" hidden="true">
       <c r="A205" t="s" s="2">
-        <v>854</v>
+        <v>849</v>
       </c>
       <c r="B205" t="s" s="2">
-        <v>854</v>
+        <v>810</v>
       </c>
       <c r="C205" s="2"/>
       <c r="D205" t="s" s="2">
@@ -27106,7 +27237,7 @@
         <v>90</v>
       </c>
       <c r="G205" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H205" t="s" s="2">
         <v>82</v>
@@ -27118,20 +27249,16 @@
         <v>82</v>
       </c>
       <c r="K205" t="s" s="2">
-        <v>439</v>
+        <v>111</v>
       </c>
       <c r="L205" t="s" s="2">
-        <v>855</v>
+        <v>198</v>
       </c>
       <c r="M205" t="s" s="2">
-        <v>856</v>
-      </c>
-      <c r="N205" t="s" s="2">
-        <v>857</v>
-      </c>
-      <c r="O205" t="s" s="2">
-        <v>858</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="N205" s="2"/>
+      <c r="O205" s="2"/>
       <c r="P205" t="s" s="2">
         <v>82</v>
       </c>
@@ -27155,55 +27282,55 @@
         <v>82</v>
       </c>
       <c r="X205" t="s" s="2">
-        <v>177</v>
+        <v>82</v>
       </c>
       <c r="Y205" t="s" s="2">
-        <v>178</v>
+        <v>82</v>
       </c>
       <c r="Z205" t="s" s="2">
-        <v>179</v>
+        <v>82</v>
       </c>
       <c r="AA205" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AB205" t="s" s="2">
-        <v>82</v>
+        <v>115</v>
       </c>
       <c r="AC205" t="s" s="2">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="AD205" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE205" t="s" s="2">
-        <v>82</v>
+        <v>117</v>
       </c>
       <c r="AF205" t="s" s="2">
-        <v>854</v>
+        <v>118</v>
       </c>
       <c r="AG205" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AH205" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI205" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ205" t="s" s="2">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="AK205" t="s" s="2">
-        <v>859</v>
+        <v>82</v>
       </c>
       <c r="AL205" t="s" s="2">
-        <v>860</v>
+        <v>82</v>
       </c>
       <c r="AM205" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN205" t="s" s="2">
-        <v>861</v>
+        <v>82</v>
       </c>
       <c r="AO205" t="s" s="2">
         <v>82</v>
@@ -27211,18 +27338,20 @@
     </row>
     <row r="206" hidden="true">
       <c r="A206" t="s" s="2">
-        <v>862</v>
+        <v>850</v>
       </c>
       <c r="B206" t="s" s="2">
-        <v>862</v>
-      </c>
-      <c r="C206" s="2"/>
+        <v>810</v>
+      </c>
+      <c r="C206" t="s" s="2">
+        <v>812</v>
+      </c>
       <c r="D206" t="s" s="2">
         <v>82</v>
       </c>
       <c r="E206" s="2"/>
       <c r="F206" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G206" t="s" s="2">
         <v>90</v>
@@ -27237,20 +27366,16 @@
         <v>82</v>
       </c>
       <c r="K206" t="s" s="2">
-        <v>599</v>
+        <v>813</v>
       </c>
       <c r="L206" t="s" s="2">
-        <v>863</v>
+        <v>814</v>
       </c>
       <c r="M206" t="s" s="2">
-        <v>864</v>
-      </c>
-      <c r="N206" t="s" s="2">
-        <v>865</v>
-      </c>
-      <c r="O206" t="s" s="2">
-        <v>866</v>
-      </c>
+        <v>815</v>
+      </c>
+      <c r="N206" s="2"/>
+      <c r="O206" s="2"/>
       <c r="P206" t="s" s="2">
         <v>82</v>
       </c>
@@ -27298,31 +27423,31 @@
         <v>82</v>
       </c>
       <c r="AF206" t="s" s="2">
-        <v>862</v>
+        <v>118</v>
       </c>
       <c r="AG206" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH206" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI206" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ206" t="s" s="2">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="AK206" t="s" s="2">
-        <v>867</v>
+        <v>82</v>
       </c>
       <c r="AL206" t="s" s="2">
-        <v>868</v>
+        <v>82</v>
       </c>
       <c r="AM206" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN206" t="s" s="2">
-        <v>869</v>
+        <v>82</v>
       </c>
       <c r="AO206" t="s" s="2">
         <v>82</v>
@@ -27330,21 +27455,21 @@
     </row>
     <row r="207" hidden="true">
       <c r="A207" t="s" s="2">
-        <v>870</v>
+        <v>851</v>
       </c>
       <c r="B207" t="s" s="2">
-        <v>870</v>
+        <v>817</v>
       </c>
       <c r="C207" s="2"/>
       <c r="D207" t="s" s="2">
-        <v>871</v>
+        <v>82</v>
       </c>
       <c r="E207" s="2"/>
       <c r="F207" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G207" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H207" t="s" s="2">
         <v>82</v>
@@ -27356,17 +27481,15 @@
         <v>82</v>
       </c>
       <c r="K207" t="s" s="2">
-        <v>872</v>
+        <v>104</v>
       </c>
       <c r="L207" t="s" s="2">
-        <v>873</v>
+        <v>105</v>
       </c>
       <c r="M207" t="s" s="2">
-        <v>874</v>
-      </c>
-      <c r="N207" t="s" s="2">
-        <v>875</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="N207" s="2"/>
       <c r="O207" s="2"/>
       <c r="P207" t="s" s="2">
         <v>82</v>
@@ -27415,31 +27538,31 @@
         <v>82</v>
       </c>
       <c r="AF207" t="s" s="2">
-        <v>870</v>
+        <v>107</v>
       </c>
       <c r="AG207" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH207" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI207" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ207" t="s" s="2">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="AK207" t="s" s="2">
-        <v>876</v>
+        <v>108</v>
       </c>
       <c r="AL207" t="s" s="2">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="AM207" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN207" t="s" s="2">
-        <v>877</v>
+        <v>82</v>
       </c>
       <c r="AO207" t="s" s="2">
         <v>82</v>
@@ -27447,10 +27570,10 @@
     </row>
     <row r="208" hidden="true">
       <c r="A208" t="s" s="2">
-        <v>878</v>
+        <v>852</v>
       </c>
       <c r="B208" t="s" s="2">
-        <v>878</v>
+        <v>819</v>
       </c>
       <c r="C208" s="2"/>
       <c r="D208" t="s" s="2">
@@ -27461,7 +27584,7 @@
         <v>80</v>
       </c>
       <c r="G208" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H208" t="s" s="2">
         <v>82</v>
@@ -27470,23 +27593,19 @@
         <v>82</v>
       </c>
       <c r="J208" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="K208" t="s" s="2">
-        <v>879</v>
+        <v>111</v>
       </c>
       <c r="L208" t="s" s="2">
-        <v>880</v>
+        <v>198</v>
       </c>
       <c r="M208" t="s" s="2">
-        <v>881</v>
-      </c>
-      <c r="N208" t="s" s="2">
-        <v>882</v>
-      </c>
-      <c r="O208" t="s" s="2">
-        <v>883</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="N208" s="2"/>
+      <c r="O208" s="2"/>
       <c r="P208" t="s" s="2">
         <v>82</v>
       </c>
@@ -27522,37 +27641,37 @@
         <v>82</v>
       </c>
       <c r="AB208" t="s" s="2">
-        <v>82</v>
+        <v>115</v>
       </c>
       <c r="AC208" t="s" s="2">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="AD208" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE208" t="s" s="2">
-        <v>82</v>
+        <v>117</v>
       </c>
       <c r="AF208" t="s" s="2">
-        <v>878</v>
+        <v>118</v>
       </c>
       <c r="AG208" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH208" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI208" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ208" t="s" s="2">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="AK208" t="s" s="2">
-        <v>838</v>
+        <v>82</v>
       </c>
       <c r="AL208" t="s" s="2">
-        <v>884</v>
+        <v>82</v>
       </c>
       <c r="AM208" t="s" s="2">
         <v>82</v>
@@ -27566,10 +27685,10 @@
     </row>
     <row r="209" hidden="true">
       <c r="A209" t="s" s="2">
-        <v>885</v>
+        <v>853</v>
       </c>
       <c r="B209" t="s" s="2">
-        <v>885</v>
+        <v>821</v>
       </c>
       <c r="C209" s="2"/>
       <c r="D209" t="s" s="2">
@@ -27577,41 +27696,39 @@
       </c>
       <c r="E209" s="2"/>
       <c r="F209" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G209" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H209" t="s" s="2">
         <v>82</v>
       </c>
       <c r="I209" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="J209" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="K209" t="s" s="2">
-        <v>770</v>
+        <v>132</v>
       </c>
       <c r="L209" t="s" s="2">
-        <v>886</v>
+        <v>225</v>
       </c>
       <c r="M209" t="s" s="2">
-        <v>887</v>
+        <v>226</v>
       </c>
       <c r="N209" t="s" s="2">
-        <v>888</v>
-      </c>
-      <c r="O209" t="s" s="2">
-        <v>889</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="O209" s="2"/>
       <c r="P209" t="s" s="2">
         <v>82</v>
       </c>
       <c r="Q209" s="2"/>
       <c r="R209" t="s" s="2">
-        <v>82</v>
+        <v>822</v>
       </c>
       <c r="S209" t="s" s="2">
         <v>82</v>
@@ -27653,25 +27770,25 @@
         <v>82</v>
       </c>
       <c r="AF209" t="s" s="2">
-        <v>885</v>
+        <v>228</v>
       </c>
       <c r="AG209" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AH209" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI209" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ209" t="s" s="2">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="AK209" t="s" s="2">
-        <v>890</v>
+        <v>196</v>
       </c>
       <c r="AL209" t="s" s="2">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="AM209" t="s" s="2">
         <v>82</v>
@@ -27685,10 +27802,10 @@
     </row>
     <row r="210" hidden="true">
       <c r="A210" t="s" s="2">
-        <v>891</v>
+        <v>854</v>
       </c>
       <c r="B210" t="s" s="2">
-        <v>891</v>
+        <v>824</v>
       </c>
       <c r="C210" s="2"/>
       <c r="D210" t="s" s="2">
@@ -27711,13 +27828,13 @@
         <v>82</v>
       </c>
       <c r="K210" t="s" s="2">
-        <v>104</v>
+        <v>173</v>
       </c>
       <c r="L210" t="s" s="2">
-        <v>105</v>
+        <v>231</v>
       </c>
       <c r="M210" t="s" s="2">
-        <v>106</v>
+        <v>232</v>
       </c>
       <c r="N210" s="2"/>
       <c r="O210" s="2"/>
@@ -27729,7 +27846,7 @@
         <v>82</v>
       </c>
       <c r="S210" t="s" s="2">
-        <v>82</v>
+        <v>845</v>
       </c>
       <c r="T210" t="s" s="2">
         <v>82</v>
@@ -27744,13 +27861,11 @@
         <v>82</v>
       </c>
       <c r="X210" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y210" t="s" s="2">
-        <v>82</v>
-      </c>
+        <v>264</v>
+      </c>
+      <c r="Y210" s="2"/>
       <c r="Z210" t="s" s="2">
-        <v>82</v>
+        <v>825</v>
       </c>
       <c r="AA210" t="s" s="2">
         <v>82</v>
@@ -27768,7 +27883,7 @@
         <v>82</v>
       </c>
       <c r="AF210" t="s" s="2">
-        <v>107</v>
+        <v>234</v>
       </c>
       <c r="AG210" t="s" s="2">
         <v>80</v>
@@ -27780,10 +27895,10 @@
         <v>82</v>
       </c>
       <c r="AJ210" t="s" s="2">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="AK210" t="s" s="2">
-        <v>108</v>
+        <v>196</v>
       </c>
       <c r="AL210" t="s" s="2">
         <v>82</v>
@@ -27800,14 +27915,14 @@
     </row>
     <row r="211" hidden="true">
       <c r="A211" t="s" s="2">
-        <v>892</v>
+        <v>855</v>
       </c>
       <c r="B211" t="s" s="2">
-        <v>892</v>
+        <v>827</v>
       </c>
       <c r="C211" s="2"/>
       <c r="D211" t="s" s="2">
-        <v>110</v>
+        <v>82</v>
       </c>
       <c r="E211" s="2"/>
       <c r="F211" t="s" s="2">
@@ -27823,21 +27938,23 @@
         <v>82</v>
       </c>
       <c r="J211" t="s" s="2">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="K211" t="s" s="2">
-        <v>111</v>
+        <v>151</v>
       </c>
       <c r="L211" t="s" s="2">
-        <v>112</v>
+        <v>828</v>
       </c>
       <c r="M211" t="s" s="2">
-        <v>113</v>
+        <v>829</v>
       </c>
       <c r="N211" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="O211" s="2"/>
+        <v>830</v>
+      </c>
+      <c r="O211" t="s" s="2">
+        <v>831</v>
+      </c>
       <c r="P211" t="s" s="2">
         <v>82</v>
       </c>
@@ -27885,7 +28002,7 @@
         <v>82</v>
       </c>
       <c r="AF211" t="s" s="2">
-        <v>118</v>
+        <v>832</v>
       </c>
       <c r="AG211" t="s" s="2">
         <v>80</v>
@@ -27897,10 +28014,10 @@
         <v>82</v>
       </c>
       <c r="AJ211" t="s" s="2">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="AK211" t="s" s="2">
-        <v>108</v>
+        <v>833</v>
       </c>
       <c r="AL211" t="s" s="2">
         <v>82</v>
@@ -27909,7 +28026,7 @@
         <v>82</v>
       </c>
       <c r="AN211" t="s" s="2">
-        <v>82</v>
+        <v>834</v>
       </c>
       <c r="AO211" t="s" s="2">
         <v>82</v>
@@ -27917,45 +28034,45 @@
     </row>
     <row r="212" hidden="true">
       <c r="A212" t="s" s="2">
-        <v>893</v>
+        <v>856</v>
       </c>
       <c r="B212" t="s" s="2">
-        <v>893</v>
+        <v>836</v>
       </c>
       <c r="C212" s="2"/>
       <c r="D212" t="s" s="2">
-        <v>790</v>
+        <v>82</v>
       </c>
       <c r="E212" s="2"/>
       <c r="F212" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G212" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H212" t="s" s="2">
         <v>82</v>
       </c>
       <c r="I212" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="J212" t="s" s="2">
         <v>91</v>
       </c>
       <c r="K212" t="s" s="2">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="L212" t="s" s="2">
-        <v>791</v>
+        <v>837</v>
       </c>
       <c r="M212" t="s" s="2">
-        <v>792</v>
+        <v>838</v>
       </c>
       <c r="N212" t="s" s="2">
-        <v>114</v>
+        <v>839</v>
       </c>
       <c r="O212" t="s" s="2">
-        <v>406</v>
+        <v>840</v>
       </c>
       <c r="P212" t="s" s="2">
         <v>82</v>
@@ -28004,22 +28121,22 @@
         <v>82</v>
       </c>
       <c r="AF212" t="s" s="2">
-        <v>793</v>
+        <v>841</v>
       </c>
       <c r="AG212" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH212" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI212" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ212" t="s" s="2">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="AK212" t="s" s="2">
-        <v>196</v>
+        <v>842</v>
       </c>
       <c r="AL212" t="s" s="2">
         <v>82</v>
@@ -28028,7 +28145,7 @@
         <v>82</v>
       </c>
       <c r="AN212" t="s" s="2">
-        <v>82</v>
+        <v>843</v>
       </c>
       <c r="AO212" t="s" s="2">
         <v>82</v>
@@ -28036,10 +28153,10 @@
     </row>
     <row r="213" hidden="true">
       <c r="A213" t="s" s="2">
-        <v>894</v>
+        <v>857</v>
       </c>
       <c r="B213" t="s" s="2">
-        <v>894</v>
+        <v>857</v>
       </c>
       <c r="C213" s="2"/>
       <c r="D213" t="s" s="2">
@@ -28047,7 +28164,7 @@
       </c>
       <c r="E213" s="2"/>
       <c r="F213" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G213" t="s" s="2">
         <v>90</v>
@@ -28059,21 +28176,21 @@
         <v>82</v>
       </c>
       <c r="J213" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="K213" t="s" s="2">
-        <v>895</v>
+        <v>608</v>
       </c>
       <c r="L213" t="s" s="2">
-        <v>896</v>
+        <v>858</v>
       </c>
       <c r="M213" t="s" s="2">
-        <v>897</v>
-      </c>
-      <c r="N213" t="s" s="2">
-        <v>898</v>
-      </c>
-      <c r="O213" s="2"/>
+        <v>859</v>
+      </c>
+      <c r="N213" s="2"/>
+      <c r="O213" t="s" s="2">
+        <v>860</v>
+      </c>
       <c r="P213" t="s" s="2">
         <v>82</v>
       </c>
@@ -28121,10 +28238,10 @@
         <v>82</v>
       </c>
       <c r="AF213" t="s" s="2">
-        <v>894</v>
+        <v>857</v>
       </c>
       <c r="AG213" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AH213" t="s" s="2">
         <v>90</v>
@@ -28136,7 +28253,7 @@
         <v>102</v>
       </c>
       <c r="AK213" t="s" s="2">
-        <v>415</v>
+        <v>614</v>
       </c>
       <c r="AL213" t="s" s="2">
         <v>108</v>
@@ -28145,7 +28262,7 @@
         <v>82</v>
       </c>
       <c r="AN213" t="s" s="2">
-        <v>899</v>
+        <v>861</v>
       </c>
       <c r="AO213" t="s" s="2">
         <v>82</v>
@@ -28153,10 +28270,10 @@
     </row>
     <row r="214" hidden="true">
       <c r="A214" t="s" s="2">
-        <v>900</v>
+        <v>862</v>
       </c>
       <c r="B214" t="s" s="2">
-        <v>900</v>
+        <v>862</v>
       </c>
       <c r="C214" s="2"/>
       <c r="D214" t="s" s="2">
@@ -28164,10 +28281,10 @@
       </c>
       <c r="E214" s="2"/>
       <c r="F214" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G214" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H214" t="s" s="2">
         <v>82</v>
@@ -28176,19 +28293,23 @@
         <v>82</v>
       </c>
       <c r="J214" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="K214" t="s" s="2">
-        <v>173</v>
+        <v>703</v>
       </c>
       <c r="L214" t="s" s="2">
-        <v>901</v>
+        <v>863</v>
       </c>
       <c r="M214" t="s" s="2">
-        <v>902</v>
-      </c>
-      <c r="N214" s="2"/>
-      <c r="O214" s="2"/>
+        <v>864</v>
+      </c>
+      <c r="N214" t="s" s="2">
+        <v>865</v>
+      </c>
+      <c r="O214" t="s" s="2">
+        <v>707</v>
+      </c>
       <c r="P214" t="s" s="2">
         <v>82</v>
       </c>
@@ -28212,13 +28333,13 @@
         <v>82</v>
       </c>
       <c r="X214" t="s" s="2">
-        <v>264</v>
+        <v>82</v>
       </c>
       <c r="Y214" t="s" s="2">
-        <v>902</v>
+        <v>82</v>
       </c>
       <c r="Z214" t="s" s="2">
-        <v>903</v>
+        <v>82</v>
       </c>
       <c r="AA214" t="s" s="2">
         <v>82</v>
@@ -28236,13 +28357,13 @@
         <v>82</v>
       </c>
       <c r="AF214" t="s" s="2">
-        <v>900</v>
+        <v>862</v>
       </c>
       <c r="AG214" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AH214" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI214" t="s" s="2">
         <v>82</v>
@@ -28251,7 +28372,7 @@
         <v>102</v>
       </c>
       <c r="AK214" t="s" s="2">
-        <v>904</v>
+        <v>708</v>
       </c>
       <c r="AL214" t="s" s="2">
         <v>108</v>
@@ -28260,14 +28381,2126 @@
         <v>82</v>
       </c>
       <c r="AN214" t="s" s="2">
-        <v>82</v>
+        <v>866</v>
       </c>
       <c r="AO214" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="215" hidden="true">
+      <c r="A215" t="s" s="2">
+        <v>867</v>
+      </c>
+      <c r="B215" t="s" s="2">
+        <v>867</v>
+      </c>
+      <c r="C215" s="2"/>
+      <c r="D215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E215" s="2"/>
+      <c r="F215" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G215" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="K215" t="s" s="2">
+        <v>868</v>
+      </c>
+      <c r="L215" t="s" s="2">
+        <v>869</v>
+      </c>
+      <c r="M215" t="s" s="2">
+        <v>870</v>
+      </c>
+      <c r="N215" s="2"/>
+      <c r="O215" t="s" s="2">
+        <v>871</v>
+      </c>
+      <c r="P215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q215" s="2"/>
+      <c r="R215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF215" t="s" s="2">
+        <v>867</v>
+      </c>
+      <c r="AG215" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH215" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ215" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK215" t="s" s="2">
+        <v>742</v>
+      </c>
+      <c r="AL215" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AM215" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN215" t="s" s="2">
+        <v>872</v>
+      </c>
+      <c r="AO215" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="216" hidden="true">
+      <c r="A216" t="s" s="2">
+        <v>873</v>
+      </c>
+      <c r="B216" t="s" s="2">
+        <v>873</v>
+      </c>
+      <c r="C216" s="2"/>
+      <c r="D216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E216" s="2"/>
+      <c r="F216" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G216" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="K216" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="L216" t="s" s="2">
+        <v>874</v>
+      </c>
+      <c r="M216" t="s" s="2">
+        <v>875</v>
+      </c>
+      <c r="N216" s="2"/>
+      <c r="O216" t="s" s="2">
+        <v>876</v>
+      </c>
+      <c r="P216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q216" s="2"/>
+      <c r="R216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X216" t="s" s="2">
+        <v>264</v>
+      </c>
+      <c r="Y216" t="s" s="2">
+        <v>877</v>
+      </c>
+      <c r="Z216" t="s" s="2">
+        <v>878</v>
+      </c>
+      <c r="AA216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF216" t="s" s="2">
+        <v>873</v>
+      </c>
+      <c r="AG216" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH216" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ216" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK216" t="s" s="2">
+        <v>717</v>
+      </c>
+      <c r="AL216" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AM216" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN216" t="s" s="2">
+        <v>879</v>
+      </c>
+      <c r="AO216" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="217" hidden="true">
+      <c r="A217" t="s" s="2">
+        <v>880</v>
+      </c>
+      <c r="B217" t="s" s="2">
+        <v>880</v>
+      </c>
+      <c r="C217" s="2"/>
+      <c r="D217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E217" s="2"/>
+      <c r="F217" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G217" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="K217" t="s" s="2">
+        <v>477</v>
+      </c>
+      <c r="L217" t="s" s="2">
+        <v>881</v>
+      </c>
+      <c r="M217" t="s" s="2">
+        <v>882</v>
+      </c>
+      <c r="N217" s="2"/>
+      <c r="O217" t="s" s="2">
+        <v>883</v>
+      </c>
+      <c r="P217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q217" s="2"/>
+      <c r="R217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF217" t="s" s="2">
+        <v>880</v>
+      </c>
+      <c r="AG217" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH217" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI217" t="s" s="2">
+        <v>884</v>
+      </c>
+      <c r="AJ217" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK217" t="s" s="2">
+        <v>885</v>
+      </c>
+      <c r="AL217" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AM217" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN217" t="s" s="2">
+        <v>886</v>
+      </c>
+      <c r="AO217" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="218" hidden="true">
+      <c r="A218" t="s" s="2">
+        <v>887</v>
+      </c>
+      <c r="B218" t="s" s="2">
+        <v>887</v>
+      </c>
+      <c r="C218" s="2"/>
+      <c r="D218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E218" s="2"/>
+      <c r="F218" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G218" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="K218" t="s" s="2">
+        <v>390</v>
+      </c>
+      <c r="L218" t="s" s="2">
+        <v>888</v>
+      </c>
+      <c r="M218" t="s" s="2">
+        <v>889</v>
+      </c>
+      <c r="N218" s="2"/>
+      <c r="O218" s="2"/>
+      <c r="P218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q218" s="2"/>
+      <c r="R218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF218" t="s" s="2">
+        <v>887</v>
+      </c>
+      <c r="AG218" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH218" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ218" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK218" t="s" s="2">
+        <v>890</v>
+      </c>
+      <c r="AL218" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AM218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN218" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO218" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="219" hidden="true">
+      <c r="A219" t="s" s="2">
+        <v>891</v>
+      </c>
+      <c r="B219" t="s" s="2">
+        <v>891</v>
+      </c>
+      <c r="C219" s="2"/>
+      <c r="D219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E219" s="2"/>
+      <c r="F219" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G219" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="K219" t="s" s="2">
+        <v>770</v>
+      </c>
+      <c r="L219" t="s" s="2">
+        <v>892</v>
+      </c>
+      <c r="M219" t="s" s="2">
+        <v>893</v>
+      </c>
+      <c r="N219" t="s" s="2">
+        <v>894</v>
+      </c>
+      <c r="O219" t="s" s="2">
+        <v>895</v>
+      </c>
+      <c r="P219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q219" s="2"/>
+      <c r="R219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF219" t="s" s="2">
+        <v>891</v>
+      </c>
+      <c r="AG219" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH219" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ219" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK219" t="s" s="2">
+        <v>896</v>
+      </c>
+      <c r="AL219" t="s" s="2">
+        <v>897</v>
+      </c>
+      <c r="AM219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN219" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO219" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="220" hidden="true">
+      <c r="A220" t="s" s="2">
+        <v>898</v>
+      </c>
+      <c r="B220" t="s" s="2">
+        <v>898</v>
+      </c>
+      <c r="C220" s="2"/>
+      <c r="D220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E220" s="2"/>
+      <c r="F220" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G220" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="K220" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="L220" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="M220" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="N220" s="2"/>
+      <c r="O220" s="2"/>
+      <c r="P220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q220" s="2"/>
+      <c r="R220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF220" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="AG220" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH220" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AK220" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AL220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AM220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN220" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO220" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="221" hidden="true">
+      <c r="A221" t="s" s="2">
+        <v>899</v>
+      </c>
+      <c r="B221" t="s" s="2">
+        <v>899</v>
+      </c>
+      <c r="C221" s="2"/>
+      <c r="D221" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="E221" s="2"/>
+      <c r="F221" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G221" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="K221" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L221" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="M221" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="N221" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="O221" s="2"/>
+      <c r="P221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q221" s="2"/>
+      <c r="R221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF221" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="AG221" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH221" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ221" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK221" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AL221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AM221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN221" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO221" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="222" hidden="true">
+      <c r="A222" t="s" s="2">
+        <v>900</v>
+      </c>
+      <c r="B222" t="s" s="2">
+        <v>900</v>
+      </c>
+      <c r="C222" s="2"/>
+      <c r="D222" t="s" s="2">
+        <v>790</v>
+      </c>
+      <c r="E222" s="2"/>
+      <c r="F222" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G222" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I222" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="J222" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="K222" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L222" t="s" s="2">
+        <v>791</v>
+      </c>
+      <c r="M222" t="s" s="2">
+        <v>792</v>
+      </c>
+      <c r="N222" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="O222" t="s" s="2">
+        <v>406</v>
+      </c>
+      <c r="P222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q222" s="2"/>
+      <c r="R222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF222" t="s" s="2">
+        <v>793</v>
+      </c>
+      <c r="AG222" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH222" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ222" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK222" t="s" s="2">
+        <v>196</v>
+      </c>
+      <c r="AL222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AM222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN222" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO222" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="223" hidden="true">
+      <c r="A223" t="s" s="2">
+        <v>901</v>
+      </c>
+      <c r="B223" t="s" s="2">
+        <v>901</v>
+      </c>
+      <c r="C223" s="2"/>
+      <c r="D223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E223" s="2"/>
+      <c r="F223" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="G223" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="K223" t="s" s="2">
+        <v>439</v>
+      </c>
+      <c r="L223" t="s" s="2">
+        <v>902</v>
+      </c>
+      <c r="M223" t="s" s="2">
+        <v>903</v>
+      </c>
+      <c r="N223" t="s" s="2">
+        <v>904</v>
+      </c>
+      <c r="O223" t="s" s="2">
+        <v>905</v>
+      </c>
+      <c r="P223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q223" s="2"/>
+      <c r="R223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X223" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="Y223" t="s" s="2">
+        <v>178</v>
+      </c>
+      <c r="Z223" t="s" s="2">
+        <v>179</v>
+      </c>
+      <c r="AA223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF223" t="s" s="2">
+        <v>901</v>
+      </c>
+      <c r="AG223" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AH223" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ223" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK223" t="s" s="2">
+        <v>906</v>
+      </c>
+      <c r="AL223" t="s" s="2">
+        <v>907</v>
+      </c>
+      <c r="AM223" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN223" t="s" s="2">
+        <v>908</v>
+      </c>
+      <c r="AO223" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="224" hidden="true">
+      <c r="A224" t="s" s="2">
+        <v>909</v>
+      </c>
+      <c r="B224" t="s" s="2">
+        <v>909</v>
+      </c>
+      <c r="C224" s="2"/>
+      <c r="D224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E224" s="2"/>
+      <c r="F224" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G224" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="K224" t="s" s="2">
+        <v>599</v>
+      </c>
+      <c r="L224" t="s" s="2">
+        <v>910</v>
+      </c>
+      <c r="M224" t="s" s="2">
+        <v>911</v>
+      </c>
+      <c r="N224" t="s" s="2">
+        <v>912</v>
+      </c>
+      <c r="O224" t="s" s="2">
+        <v>913</v>
+      </c>
+      <c r="P224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q224" s="2"/>
+      <c r="R224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF224" t="s" s="2">
+        <v>909</v>
+      </c>
+      <c r="AG224" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH224" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ224" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK224" t="s" s="2">
+        <v>914</v>
+      </c>
+      <c r="AL224" t="s" s="2">
+        <v>915</v>
+      </c>
+      <c r="AM224" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN224" t="s" s="2">
+        <v>916</v>
+      </c>
+      <c r="AO224" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="225" hidden="true">
+      <c r="A225" t="s" s="2">
+        <v>917</v>
+      </c>
+      <c r="B225" t="s" s="2">
+        <v>917</v>
+      </c>
+      <c r="C225" s="2"/>
+      <c r="D225" t="s" s="2">
+        <v>918</v>
+      </c>
+      <c r="E225" s="2"/>
+      <c r="F225" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G225" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="K225" t="s" s="2">
+        <v>919</v>
+      </c>
+      <c r="L225" t="s" s="2">
+        <v>920</v>
+      </c>
+      <c r="M225" t="s" s="2">
+        <v>921</v>
+      </c>
+      <c r="N225" t="s" s="2">
+        <v>922</v>
+      </c>
+      <c r="O225" s="2"/>
+      <c r="P225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q225" s="2"/>
+      <c r="R225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF225" t="s" s="2">
+        <v>917</v>
+      </c>
+      <c r="AG225" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH225" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ225" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK225" t="s" s="2">
+        <v>923</v>
+      </c>
+      <c r="AL225" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AM225" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN225" t="s" s="2">
+        <v>924</v>
+      </c>
+      <c r="AO225" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="226" hidden="true">
+      <c r="A226" t="s" s="2">
+        <v>925</v>
+      </c>
+      <c r="B226" t="s" s="2">
+        <v>925</v>
+      </c>
+      <c r="C226" s="2"/>
+      <c r="D226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E226" s="2"/>
+      <c r="F226" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G226" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J226" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="K226" t="s" s="2">
+        <v>926</v>
+      </c>
+      <c r="L226" t="s" s="2">
+        <v>927</v>
+      </c>
+      <c r="M226" t="s" s="2">
+        <v>928</v>
+      </c>
+      <c r="N226" t="s" s="2">
+        <v>929</v>
+      </c>
+      <c r="O226" t="s" s="2">
+        <v>930</v>
+      </c>
+      <c r="P226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q226" s="2"/>
+      <c r="R226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF226" t="s" s="2">
+        <v>925</v>
+      </c>
+      <c r="AG226" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH226" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ226" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK226" t="s" s="2">
+        <v>885</v>
+      </c>
+      <c r="AL226" t="s" s="2">
+        <v>931</v>
+      </c>
+      <c r="AM226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN226" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO226" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="227" hidden="true">
+      <c r="A227" t="s" s="2">
+        <v>932</v>
+      </c>
+      <c r="B227" t="s" s="2">
+        <v>932</v>
+      </c>
+      <c r="C227" s="2"/>
+      <c r="D227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E227" s="2"/>
+      <c r="F227" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G227" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I227" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="J227" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="K227" t="s" s="2">
+        <v>770</v>
+      </c>
+      <c r="L227" t="s" s="2">
+        <v>933</v>
+      </c>
+      <c r="M227" t="s" s="2">
+        <v>934</v>
+      </c>
+      <c r="N227" t="s" s="2">
+        <v>935</v>
+      </c>
+      <c r="O227" t="s" s="2">
+        <v>936</v>
+      </c>
+      <c r="P227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q227" s="2"/>
+      <c r="R227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF227" t="s" s="2">
+        <v>932</v>
+      </c>
+      <c r="AG227" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH227" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ227" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK227" t="s" s="2">
+        <v>937</v>
+      </c>
+      <c r="AL227" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AM227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN227" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO227" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="228" hidden="true">
+      <c r="A228" t="s" s="2">
+        <v>938</v>
+      </c>
+      <c r="B228" t="s" s="2">
+        <v>938</v>
+      </c>
+      <c r="C228" s="2"/>
+      <c r="D228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E228" s="2"/>
+      <c r="F228" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G228" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="K228" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="L228" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="M228" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="N228" s="2"/>
+      <c r="O228" s="2"/>
+      <c r="P228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q228" s="2"/>
+      <c r="R228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF228" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="AG228" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH228" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AK228" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AL228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AM228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN228" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO228" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="229" hidden="true">
+      <c r="A229" t="s" s="2">
+        <v>939</v>
+      </c>
+      <c r="B229" t="s" s="2">
+        <v>939</v>
+      </c>
+      <c r="C229" s="2"/>
+      <c r="D229" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="E229" s="2"/>
+      <c r="F229" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G229" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="K229" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L229" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="M229" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="N229" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="O229" s="2"/>
+      <c r="P229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q229" s="2"/>
+      <c r="R229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF229" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="AG229" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH229" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ229" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK229" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AL229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AM229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN229" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO229" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="230" hidden="true">
+      <c r="A230" t="s" s="2">
+        <v>940</v>
+      </c>
+      <c r="B230" t="s" s="2">
+        <v>940</v>
+      </c>
+      <c r="C230" s="2"/>
+      <c r="D230" t="s" s="2">
+        <v>790</v>
+      </c>
+      <c r="E230" s="2"/>
+      <c r="F230" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G230" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I230" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="J230" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="K230" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L230" t="s" s="2">
+        <v>791</v>
+      </c>
+      <c r="M230" t="s" s="2">
+        <v>792</v>
+      </c>
+      <c r="N230" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="O230" t="s" s="2">
+        <v>406</v>
+      </c>
+      <c r="P230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q230" s="2"/>
+      <c r="R230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF230" t="s" s="2">
+        <v>793</v>
+      </c>
+      <c r="AG230" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH230" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ230" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK230" t="s" s="2">
+        <v>196</v>
+      </c>
+      <c r="AL230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AM230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN230" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO230" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="231" hidden="true">
+      <c r="A231" t="s" s="2">
+        <v>941</v>
+      </c>
+      <c r="B231" t="s" s="2">
+        <v>941</v>
+      </c>
+      <c r="C231" s="2"/>
+      <c r="D231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E231" s="2"/>
+      <c r="F231" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="G231" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J231" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="K231" t="s" s="2">
+        <v>942</v>
+      </c>
+      <c r="L231" t="s" s="2">
+        <v>943</v>
+      </c>
+      <c r="M231" t="s" s="2">
+        <v>944</v>
+      </c>
+      <c r="N231" t="s" s="2">
+        <v>945</v>
+      </c>
+      <c r="O231" s="2"/>
+      <c r="P231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q231" s="2"/>
+      <c r="R231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF231" t="s" s="2">
+        <v>941</v>
+      </c>
+      <c r="AG231" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AH231" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ231" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK231" t="s" s="2">
+        <v>415</v>
+      </c>
+      <c r="AL231" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AM231" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN231" t="s" s="2">
+        <v>946</v>
+      </c>
+      <c r="AO231" t="s" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="232" hidden="true">
+      <c r="A232" t="s" s="2">
+        <v>947</v>
+      </c>
+      <c r="B232" t="s" s="2">
+        <v>947</v>
+      </c>
+      <c r="C232" s="2"/>
+      <c r="D232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E232" s="2"/>
+      <c r="F232" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="G232" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="I232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J232" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="K232" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="L232" t="s" s="2">
+        <v>948</v>
+      </c>
+      <c r="M232" t="s" s="2">
+        <v>949</v>
+      </c>
+      <c r="N232" s="2"/>
+      <c r="O232" s="2"/>
+      <c r="P232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Q232" s="2"/>
+      <c r="R232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X232" t="s" s="2">
+        <v>264</v>
+      </c>
+      <c r="Y232" t="s" s="2">
+        <v>949</v>
+      </c>
+      <c r="Z232" t="s" s="2">
+        <v>950</v>
+      </c>
+      <c r="AA232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF232" t="s" s="2">
+        <v>947</v>
+      </c>
+      <c r="AG232" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AH232" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ232" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK232" t="s" s="2">
+        <v>951</v>
+      </c>
+      <c r="AL232" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AM232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN232" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO232" t="s" s="2">
         <v>82</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AO214">
+  <autoFilter ref="A1:AO232">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -28277,7 +30510,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI213">
+  <conditionalFormatting sqref="A2:AI231">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>